<commit_message>
First Working Version Creating LLRs
</commit_message>
<xml_diff>
--- a/Requirements/High Level Requirements/Excel/High Level Requirements_1.xlsx
+++ b/Requirements/High Level Requirements/Excel/High Level Requirements_1.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="45">
   <si>
     <t>Cathegory</t>
   </si>
@@ -71,6 +71,105 @@
   </si>
   <si>
     <t>Example Description</t>
+  </si>
+  <si>
+    <t>FR</t>
+  </si>
+  <si>
+    <t>Explore Maze</t>
+  </si>
+  <si>
+    <t>Robot shall autonomously explore an unknown maze</t>
+  </si>
+  <si>
+    <t>Wall Detection</t>
+  </si>
+  <si>
+    <t>Robot shall detect and avoid walls</t>
+  </si>
+  <si>
+    <t>MAP</t>
+  </si>
+  <si>
+    <t>Create Map</t>
+  </si>
+  <si>
+    <t>Robot shall create an internal representation of the maze</t>
+  </si>
+  <si>
+    <t>Cell Clasification</t>
+  </si>
+  <si>
+    <t>Robot shall distinguish between free, blocked, and unknown areas</t>
+  </si>
+  <si>
+    <t>NFR</t>
+  </si>
+  <si>
+    <t>Time Constraint</t>
+  </si>
+  <si>
+    <t>Robot shall complete mapping of the maze within 5 minutes</t>
+  </si>
+  <si>
+    <t>PLAN</t>
+  </si>
+  <si>
+    <t>Path Planning</t>
+  </si>
+  <si>
+    <t>Robot shall compute an optimal path to the target</t>
+  </si>
+  <si>
+    <t>RUN</t>
+  </si>
+  <si>
+    <t>Return to Start</t>
+  </si>
+  <si>
+    <t>Robot shall return to start after the exploration is done</t>
+  </si>
+  <si>
+    <t>Second Run</t>
+  </si>
+  <si>
+    <t>Robot shall perform a second run after exploration</t>
+  </si>
+  <si>
+    <t>Efficient Path Execution</t>
+  </si>
+  <si>
+    <t>Second run shall follow the most efficient path to the target</t>
+  </si>
+  <si>
+    <t>RELIAB</t>
+  </si>
+  <si>
+    <t>Collision Avoidance</t>
+  </si>
+  <si>
+    <t>The robot shall not collide with walls</t>
+  </si>
+  <si>
+    <t>Fault Tolerance</t>
+  </si>
+  <si>
+    <t>The robot shall be able to handle faulty sensor data</t>
+  </si>
+  <si>
+    <t>INTERF</t>
+  </si>
+  <si>
+    <t>Sensor Processing</t>
+  </si>
+  <si>
+    <t>The system shall be able to process sensor data defined in the sensor data interface description</t>
+  </si>
+  <si>
+    <t>Actuator Control</t>
+  </si>
+  <si>
+    <t>The system shall be able to send control commands to actuators with commands specified in motor interface description</t>
   </si>
 </sst>
 </file>
@@ -407,607 +506,841 @@
         <v>11</v>
       </c>
       <c r="H2" s="4" t="str">
-        <f t="shared" ref="H2:H102" si="1">CONCATENATE("HL--", A2,"--",B2,".",C2,)</f>
+        <f t="shared" ref="H2:H4" si="1">CONCATENATE("HL--", A2,"--",B2,".",C2,)</f>
         <v>HL--EXPL--1.1</v>
       </c>
     </row>
     <row r="3">
+      <c r="A3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="C3" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>14</v>
+      </c>
       <c r="H3" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>HL----.</v>
+        <v>HL--EXPL--1.2</v>
       </c>
     </row>
     <row r="4">
+      <c r="A4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="C4" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="H4" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>HL----.</v>
+        <v>HL--EXPL--1.3</v>
       </c>
     </row>
     <row r="5">
+      <c r="A5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="C5" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="H5" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>HL----.</v>
+        <f>CONCATENATE("HL--", #REF!,"--",#REF!,".",#REF!,)</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="6">
+      <c r="A6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="C6" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>21</v>
+      </c>
       <c r="H6" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>HL----.</v>
+        <f t="shared" ref="H6:H8" si="2">CONCATENATE("HL--", A5,"--",B5,".",C5,)</f>
+        <v>HL--MAP--2.1</v>
       </c>
     </row>
     <row r="7">
+      <c r="A7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="C7" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="H7" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>HL----.</v>
+        <f t="shared" si="2"/>
+        <v>HL--MAP--2.2</v>
       </c>
     </row>
     <row r="8">
+      <c r="A8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="C8" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>27</v>
+      </c>
       <c r="H8" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>HL----.</v>
+        <f t="shared" si="2"/>
+        <v>HL--MAP--2.3</v>
       </c>
     </row>
     <row r="9">
+      <c r="A9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="C9" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>30</v>
+      </c>
       <c r="H9" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>HL----.</v>
+        <f>CONCATENATE("HL--", #REF!,"--",#REF!,".",#REF!,)</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="10">
+      <c r="A10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="C10" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="H10" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>HL----.</v>
+        <f>CONCATENATE("HL--", A8,"--",B8,".",C8,)</f>
+        <v>HL--PLAN--3.1</v>
       </c>
     </row>
     <row r="11">
+      <c r="A11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="C11" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>34</v>
+      </c>
       <c r="H11" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>HL----.</v>
+        <f>CONCATENATE("HL--", #REF!,"--",#REF!,".",#REF!,)</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="12">
+      <c r="A12" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="C12" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>37</v>
+      </c>
       <c r="H12" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>HL----.</v>
+        <f t="shared" ref="H12:H13" si="3">CONCATENATE("HL--", A10,"--",B10,".",C10,)</f>
+        <v>HL--RUN--4.2</v>
       </c>
     </row>
     <row r="13">
+      <c r="A13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="C13" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>39</v>
+      </c>
       <c r="H13" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>HL----.</v>
+        <f t="shared" si="3"/>
+        <v>HL--RUN--4.3</v>
       </c>
     </row>
     <row r="14">
+      <c r="A14" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="C14" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>42</v>
+      </c>
       <c r="H14" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>HL----.</v>
+        <f>CONCATENATE("HL--", #REF!,"--",#REF!,".",#REF!,)</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="15">
+      <c r="A15" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="C15" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>44</v>
+      </c>
       <c r="H15" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>HL----.</v>
+        <f t="shared" ref="H15:H16" si="4">CONCATENATE("HL--", A12,"--",B12,".",C12,)</f>
+        <v>HL--RELIAB--5.1</v>
       </c>
     </row>
     <row r="16">
       <c r="H16" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>HL----.</v>
+        <f t="shared" si="4"/>
+        <v>HL--RELIAB--5.2</v>
       </c>
     </row>
     <row r="17">
       <c r="H17" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f>CONCATENATE("HL--", A18,"--",B18,".",C18,)</f>
         <v>HL----.</v>
       </c>
     </row>
     <row r="18">
       <c r="H18" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>HL----.</v>
+        <f t="shared" ref="H18:H19" si="5">CONCATENATE("HL--", A14,"--",B14,".",C14,)</f>
+        <v>HL--INTERF--6.1</v>
       </c>
     </row>
     <row r="19">
       <c r="H19" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>HL----.</v>
+        <f t="shared" si="5"/>
+        <v>HL--INTERF--6.2</v>
       </c>
     </row>
     <row r="20">
       <c r="H20" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>HL----.</v>
+        <f>CONCATENATE("HL--", #REF!,"--",#REF!,".",#REF!,)</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="21">
       <c r="H21" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="H21:H102" si="6">CONCATENATE("HL--", A21,"--",B21,".",C21,)</f>
         <v>HL----.</v>
       </c>
     </row>
     <row r="22">
       <c r="H22" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="23">
       <c r="H23" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="24">
       <c r="H24" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="25">
       <c r="H25" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="26">
       <c r="H26" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="27">
       <c r="H27" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="28">
       <c r="H28" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="29">
       <c r="H29" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="30">
       <c r="H30" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="31">
       <c r="H31" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="32">
       <c r="H32" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="33">
       <c r="H33" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="34">
       <c r="H34" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="35">
       <c r="H35" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="36">
       <c r="H36" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="37">
       <c r="H37" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="38">
       <c r="H38" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="39">
       <c r="H39" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="40">
       <c r="H40" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="41">
       <c r="H41" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="42">
       <c r="H42" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="43">
       <c r="H43" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="44">
       <c r="H44" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="45">
       <c r="H45" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="46">
       <c r="H46" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="47">
       <c r="H47" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="48">
       <c r="H48" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="49">
       <c r="H49" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="50">
       <c r="H50" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="51">
       <c r="H51" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="52">
       <c r="H52" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="53">
       <c r="H53" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="54">
       <c r="H54" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="55">
       <c r="H55" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="56">
       <c r="H56" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="57">
       <c r="H57" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="58">
       <c r="H58" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="59">
       <c r="H59" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="60">
       <c r="H60" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="61">
       <c r="H61" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="62">
       <c r="H62" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="63">
       <c r="H63" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="64">
       <c r="H64" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="65">
       <c r="H65" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="66">
       <c r="H66" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="67">
       <c r="H67" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="68">
       <c r="H68" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="69">
       <c r="H69" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="70">
       <c r="H70" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="71">
       <c r="H71" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="72">
       <c r="H72" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="73">
       <c r="H73" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="74">
       <c r="H74" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="75">
       <c r="H75" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="76">
       <c r="H76" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="77">
       <c r="H77" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="78">
       <c r="H78" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="79">
       <c r="H79" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="80">
       <c r="H80" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="81">
       <c r="H81" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="82">
       <c r="H82" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="83">
       <c r="H83" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="84">
       <c r="H84" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="85">
       <c r="H85" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="86">
       <c r="H86" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="87">
       <c r="H87" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="88">
       <c r="H88" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="89">
       <c r="H89" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="90">
       <c r="H90" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="91">
       <c r="H91" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="92">
       <c r="H92" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="93">
       <c r="H93" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="94">
       <c r="H94" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="95">
       <c r="H95" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="96">
       <c r="H96" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="97">
       <c r="H97" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="98">
       <c r="H98" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="99">
       <c r="H99" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="100">
       <c r="H100" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="101">
       <c r="H101" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>
     <row r="102">
       <c r="H102" s="4" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="6"/>
         <v>HL----.</v>
       </c>
     </row>

</xml_diff>